<commit_message>
Day 2 Deliverables updated
</commit_message>
<xml_diff>
--- a/Anumoy_Pathak_RedBus/Bus_Seat_Booking_Defect_Report.xlsx
+++ b/Anumoy_Pathak_RedBus/Bus_Seat_Booking_Defect_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d6a5426fd29e00d/Desktop/Anumoy_Pathak_RedBus/Anumoy_Pathak_RedBus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d6a5426fd29e00d/Desktop/Anumoy_Pathak_RedBus - Backup/Anumoy_Pathak_RedBus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_F25DC773A252ABDACC104866F95B43925ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA5A859D-7E5F-428F-AA66-ED60DEBA5F68}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_F25DC773A252ABDACC104866F95B43925ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA3C17A6-8240-459E-B23B-60C6F1E70401}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5328" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,9 +45,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>abc@capgemini.com</t>
-  </si>
-  <si>
     <t>To do</t>
   </si>
   <si>
@@ -58,6 +55,9 @@
   </si>
   <si>
     <t>Boarding &amp; Dropping</t>
+  </si>
+  <si>
+    <t>Dev Team</t>
   </si>
   <si>
     <t>Medium</t>
@@ -136,10 +136,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -438,22 +434,22 @@
     </row>
     <row r="2" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>